<commit_message>
WIP: ECU splice point (4 bussed DT plugs), ECU ground alone to the NEG bar, CAN-node grounds to the NEG bar
</commit_message>
<xml_diff>
--- a/docs/harness/wirelist/CAN-wirelist.xlsx
+++ b/docs/harness/wirelist/CAN-wirelist.xlsx
@@ -3916,7 +3916,7 @@
       </c>
       <c r="M27" s="29" t="inlineStr">
         <is>
-          <t>Ground point IF, I/P brace RH (EWD ground point IF, p.42)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="N27" s="28" t="inlineStr"/>
@@ -3925,7 +3925,11 @@
           <t>Cluster ground</t>
         </is>
       </c>
-      <c r="P27" s="29" t="inlineStr"/>
+      <c r="P27" s="29" t="inlineStr">
+        <is>
+          <t>M8 ring lug on the POWER box battery-negative bar (R213 / R217: a CAN node never on chassis); runs with the CAN trunk to the ECU, then with the ECU harness to the glove box</t>
+        </is>
+      </c>
       <c r="Q27" s="30" t="inlineStr">
         <is>
           <t>GND.t_cluster_gnd</t>
@@ -3933,7 +3937,7 @@
       </c>
       <c r="R27" s="31" t="inlineStr">
         <is>
-          <t>Chassis GND (Ground point IF, I/P brace RH (EWD ground point IF, p.42))</t>
+          <t>Chassis GND (POWER box NEG bar M8 stud (glove box))</t>
         </is>
       </c>
       <c r="S27" s="32" t="inlineStr"/>
@@ -3953,7 +3957,7 @@
         </is>
       </c>
       <c r="Y27" s="34" t="n">
-        <v>1320</v>
+        <v>1600</v>
       </c>
       <c r="Z27" s="35" t="inlineStr"/>
       <c r="AA27" s="36" t="inlineStr"/>
@@ -3970,7 +3974,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG27" s="38" t="inlineStr"/>
+      <c r="AG27" s="38" t="inlineStr">
+        <is>
+          <t>est length to the glove-box NEG bar (was factory ground point IF)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="39" t="inlineStr">
@@ -4023,7 +4031,7 @@
       </c>
       <c r="M28" s="45" t="inlineStr">
         <is>
-          <t>Ground point IF, I/P brace RH (EWD ground point IF, p.42)</t>
+          <t>POWER box NEG bar M8 stud (glove box)</t>
         </is>
       </c>
       <c r="N28" s="44" t="inlineStr"/>
@@ -4032,7 +4040,11 @@
           <t>RealDash Pi ground</t>
         </is>
       </c>
-      <c r="P28" s="45" t="inlineStr"/>
+      <c r="P28" s="45" t="inlineStr">
+        <is>
+          <t>M8 ring lug on the POWER box battery-negative bar (R213 / R217: a CAN node never on chassis); runs with the CAN trunk to the ECU, then with the ECU harness to the glove box</t>
+        </is>
+      </c>
       <c r="Q28" s="46" t="inlineStr">
         <is>
           <t>GND.t_cluster_gnd</t>
@@ -4040,7 +4052,7 @@
       </c>
       <c r="R28" s="47" t="inlineStr">
         <is>
-          <t>Chassis GND (Ground point IF, I/P brace RH (EWD ground point IF, p.42))</t>
+          <t>Chassis GND (POWER box NEG bar M8 stud (glove box))</t>
         </is>
       </c>
       <c r="S28" s="48" t="inlineStr"/>
@@ -4060,7 +4072,7 @@
         </is>
       </c>
       <c r="Y28" s="50" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="Z28" s="51" t="inlineStr"/>
       <c r="AA28" s="52" t="inlineStr"/>
@@ -4077,7 +4089,11 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AG28" s="54" t="inlineStr"/>
+      <c r="AG28" s="54" t="inlineStr">
+        <is>
+          <t>est length to the glove-box NEG bar (was factory ground point IF)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="23" t="inlineStr"/>

</xml_diff>